<commit_message>
Daily recap, matchup updates, learning and research 2026-08-19
</commit_message>
<xml_diff>
--- a/data/k-props/2026-08-19.xlsx
+++ b/data/k-props/2026-08-19.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="96">
   <si>
     <t>date</t>
   </si>
@@ -145,22 +145,34 @@
     <t>lineup_unweighted_30d_posted</t>
   </si>
   <si>
+    <t>U</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>&lt;6</t>
+  </si>
+  <si>
+    <t>Michael King</t>
+  </si>
+  <si>
+    <t>San Diego Padres @ New York Mets</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>Robert Stock</t>
+  </si>
+  <si>
+    <t>Limited starter</t>
+  </si>
+  <si>
+    <t>O</t>
+  </si>
+  <si>
     <t/>
-  </si>
-  <si>
-    <t>&lt;6</t>
-  </si>
-  <si>
-    <t>Michael King</t>
-  </si>
-  <si>
-    <t>San Diego Padres @ New York Mets</t>
-  </si>
-  <si>
-    <t>Robert Stock</t>
-  </si>
-  <si>
-    <t>Limited starter</t>
   </si>
   <si>
     <t>Taj Bradley</t>
@@ -868,17 +880,23 @@
       <c r="Y2">
         <v>0.9157</v>
       </c>
+      <c r="Z2">
+        <v>5</v>
+      </c>
       <c r="AA2" t="s">
         <v>44</v>
       </c>
+      <c r="AB2">
+        <v>-1.46</v>
+      </c>
       <c r="AC2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD2">
         <v>5.04</v>
       </c>
       <c r="AE2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF2">
         <v>0.3009</v>
@@ -888,6 +906,18 @@
       </c>
       <c r="AH2">
         <v>0</v>
+      </c>
+      <c r="AI2">
+        <v>-0.04</v>
+      </c>
+      <c r="AJ2">
+        <v>0.04</v>
+      </c>
+      <c r="AK2">
+        <v>-0.04</v>
+      </c>
+      <c r="AL2">
+        <v>0.04</v>
       </c>
       <c r="AM2">
         <v>5.04</v>
@@ -898,7 +928,7 @@
         <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C3">
         <v>4.5</v>
@@ -910,7 +940,7 @@
         <v>-165</v>
       </c>
       <c r="F3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G3">
         <v>823587</v>
@@ -969,17 +999,23 @@
       <c r="Y3">
         <v>0.9921</v>
       </c>
+      <c r="Z3">
+        <v>4</v>
+      </c>
       <c r="AA3" t="s">
         <v>44</v>
       </c>
+      <c r="AB3">
+        <v>0.73</v>
+      </c>
       <c r="AC3" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="AD3">
         <v>5.23</v>
       </c>
       <c r="AE3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF3">
         <v>0.2099</v>
@@ -989,6 +1025,18 @@
       </c>
       <c r="AH3">
         <v>0</v>
+      </c>
+      <c r="AI3">
+        <v>-1.23</v>
+      </c>
+      <c r="AJ3">
+        <v>1.23</v>
+      </c>
+      <c r="AK3">
+        <v>-1.23</v>
+      </c>
+      <c r="AL3">
+        <v>1.23</v>
       </c>
       <c r="AM3">
         <v>5.23</v>
@@ -999,7 +1047,7 @@
         <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C4">
         <v>3.5</v>
@@ -1011,13 +1059,13 @@
         <v>120</v>
       </c>
       <c r="F4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G4">
         <v>823587</v>
       </c>
       <c r="H4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="I4">
         <v>4.2</v>
@@ -1070,17 +1118,23 @@
       <c r="Y4">
         <v>1.0272</v>
       </c>
+      <c r="Z4">
+        <v>6</v>
+      </c>
       <c r="AA4" t="s">
-        <v>44</v>
+        <v>52</v>
+      </c>
+      <c r="AB4">
+        <v>0.59</v>
       </c>
       <c r="AC4" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="AD4">
         <v>4.09</v>
       </c>
       <c r="AE4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF4">
         <v>0.2346</v>
@@ -1090,6 +1144,18 @@
       </c>
       <c r="AH4">
         <v>0</v>
+      </c>
+      <c r="AI4">
+        <v>1.91</v>
+      </c>
+      <c r="AJ4">
+        <v>1.91</v>
+      </c>
+      <c r="AK4">
+        <v>1.91</v>
+      </c>
+      <c r="AL4">
+        <v>1.91</v>
       </c>
       <c r="AM4">
         <v>4.09</v>
@@ -1100,7 +1166,7 @@
         <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C5">
         <v>5.5</v>
@@ -1112,7 +1178,7 @@
         <v>108</v>
       </c>
       <c r="F5" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G5">
         <v>823664</v>
@@ -1171,17 +1237,23 @@
       <c r="Y5">
         <v>1.0473</v>
       </c>
+      <c r="Z5">
+        <v>7</v>
+      </c>
       <c r="AA5" t="s">
-        <v>44</v>
+        <v>52</v>
+      </c>
+      <c r="AB5">
+        <v>1.41</v>
       </c>
       <c r="AC5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD5">
         <v>6.91</v>
       </c>
       <c r="AE5" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="AF5">
         <v>0.2571</v>
@@ -1191,6 +1263,18 @@
       </c>
       <c r="AH5">
         <v>0</v>
+      </c>
+      <c r="AI5">
+        <v>0.09</v>
+      </c>
+      <c r="AJ5">
+        <v>0.09</v>
+      </c>
+      <c r="AK5">
+        <v>0.09</v>
+      </c>
+      <c r="AL5">
+        <v>0.09</v>
       </c>
       <c r="AM5">
         <v>6.91</v>
@@ -1201,16 +1285,16 @@
         <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="F6" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="G6">
         <v>824640</v>
       </c>
       <c r="H6" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="I6">
         <v>2.1</v>
@@ -1264,16 +1348,16 @@
         <v>0.8952</v>
       </c>
       <c r="AA6" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="AC6" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="AD6">
         <v>1.7</v>
       </c>
       <c r="AE6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF6">
         <v>0.2318</v>
@@ -1293,7 +1377,7 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C7">
         <v>3.5</v>
@@ -1305,7 +1389,7 @@
         <v>-170</v>
       </c>
       <c r="F7" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="G7">
         <v>824640</v>
@@ -1364,17 +1448,23 @@
       <c r="Y7">
         <v>1.0504</v>
       </c>
+      <c r="Z7">
+        <v>1</v>
+      </c>
       <c r="AA7" t="s">
         <v>44</v>
       </c>
+      <c r="AB7">
+        <v>1.35</v>
+      </c>
       <c r="AC7" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="AD7">
         <v>4.85</v>
       </c>
       <c r="AE7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF7">
         <v>0.1773</v>
@@ -1384,6 +1474,18 @@
       </c>
       <c r="AH7">
         <v>0</v>
+      </c>
+      <c r="AI7">
+        <v>-3.85</v>
+      </c>
+      <c r="AJ7">
+        <v>3.85</v>
+      </c>
+      <c r="AK7">
+        <v>-3.85</v>
+      </c>
+      <c r="AL7">
+        <v>3.85</v>
       </c>
       <c r="AM7">
         <v>4.85</v>
@@ -1394,7 +1496,7 @@
         <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C8">
         <v>8.5</v>
@@ -1406,7 +1508,7 @@
         <v>-185</v>
       </c>
       <c r="F8" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G8">
         <v>824722</v>
@@ -1465,17 +1567,23 @@
       <c r="Y8">
         <v>1.0088</v>
       </c>
+      <c r="Z8">
+        <v>8</v>
+      </c>
       <c r="AA8" t="s">
         <v>44</v>
       </c>
+      <c r="AB8">
+        <v>-4.77</v>
+      </c>
       <c r="AC8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD8">
         <v>3.73</v>
       </c>
       <c r="AE8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF8">
         <v>0.1803</v>
@@ -1485,6 +1593,18 @@
       </c>
       <c r="AH8">
         <v>0</v>
+      </c>
+      <c r="AI8">
+        <v>4.27</v>
+      </c>
+      <c r="AJ8">
+        <v>4.27</v>
+      </c>
+      <c r="AK8">
+        <v>4.27</v>
+      </c>
+      <c r="AL8">
+        <v>4.27</v>
       </c>
       <c r="AM8">
         <v>3.73</v>
@@ -1495,7 +1615,7 @@
         <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C9">
         <v>5.5</v>
@@ -1507,7 +1627,7 @@
         <v>102</v>
       </c>
       <c r="F9" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G9">
         <v>824722</v>
@@ -1566,17 +1686,23 @@
       <c r="Y9">
         <v>0.88</v>
       </c>
+      <c r="Z9">
+        <v>6</v>
+      </c>
       <c r="AA9" t="s">
-        <v>44</v>
+        <v>52</v>
+      </c>
+      <c r="AB9">
+        <v>0.82</v>
       </c>
       <c r="AC9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD9">
         <v>6.32</v>
       </c>
       <c r="AE9" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="AF9">
         <v>0.2958</v>
@@ -1586,6 +1712,18 @@
       </c>
       <c r="AH9">
         <v>0</v>
+      </c>
+      <c r="AI9">
+        <v>-0.32</v>
+      </c>
+      <c r="AJ9">
+        <v>0.32</v>
+      </c>
+      <c r="AK9">
+        <v>-0.32</v>
+      </c>
+      <c r="AL9">
+        <v>0.32</v>
       </c>
       <c r="AM9">
         <v>6.32</v>
@@ -1596,7 +1734,7 @@
         <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C10">
         <v>4.5</v>
@@ -1608,7 +1746,7 @@
         <v>-145</v>
       </c>
       <c r="F10" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="G10">
         <v>823424</v>
@@ -1667,17 +1805,23 @@
       <c r="Y10">
         <v>0.9247</v>
       </c>
+      <c r="Z10">
+        <v>1</v>
+      </c>
       <c r="AA10" t="s">
         <v>44</v>
       </c>
+      <c r="AB10">
+        <v>-0.89</v>
+      </c>
       <c r="AC10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD10">
         <v>3.61</v>
       </c>
       <c r="AE10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF10">
         <v>0.1754</v>
@@ -1687,6 +1831,18 @@
       </c>
       <c r="AH10">
         <v>0</v>
+      </c>
+      <c r="AI10">
+        <v>-2.61</v>
+      </c>
+      <c r="AJ10">
+        <v>2.61</v>
+      </c>
+      <c r="AK10">
+        <v>-2.61</v>
+      </c>
+      <c r="AL10">
+        <v>2.61</v>
       </c>
       <c r="AM10">
         <v>3.61</v>
@@ -1697,7 +1853,7 @@
         <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C11">
         <v>5.5</v>
@@ -1709,7 +1865,7 @@
         <v>108</v>
       </c>
       <c r="F11" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="G11">
         <v>823424</v>
@@ -1768,17 +1924,23 @@
       <c r="Y11">
         <v>0.9512</v>
       </c>
+      <c r="Z11">
+        <v>8</v>
+      </c>
       <c r="AA11" t="s">
-        <v>44</v>
+        <v>52</v>
+      </c>
+      <c r="AB11">
+        <v>0.47</v>
       </c>
       <c r="AC11" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="AD11">
         <v>5.97</v>
       </c>
       <c r="AE11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF11">
         <v>0.2561</v>
@@ -1788,6 +1950,18 @@
       </c>
       <c r="AH11">
         <v>0</v>
+      </c>
+      <c r="AI11">
+        <v>2.03</v>
+      </c>
+      <c r="AJ11">
+        <v>2.03</v>
+      </c>
+      <c r="AK11">
+        <v>2.03</v>
+      </c>
+      <c r="AL11">
+        <v>2.03</v>
       </c>
       <c r="AM11">
         <v>5.97</v>
@@ -1798,7 +1972,7 @@
         <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C12">
         <v>5.5</v>
@@ -1810,7 +1984,7 @@
         <v>-147</v>
       </c>
       <c r="F12" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G12">
         <v>824801</v>
@@ -1869,17 +2043,23 @@
       <c r="Y12">
         <v>1.0727</v>
       </c>
+      <c r="Z12">
+        <v>5</v>
+      </c>
       <c r="AA12" t="s">
         <v>44</v>
       </c>
+      <c r="AB12">
+        <v>0.4</v>
+      </c>
       <c r="AC12" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="AD12">
         <v>5.9</v>
       </c>
       <c r="AE12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF12">
         <v>0.2386</v>
@@ -1889,6 +2069,18 @@
       </c>
       <c r="AH12">
         <v>0</v>
+      </c>
+      <c r="AI12">
+        <v>-0.9</v>
+      </c>
+      <c r="AJ12">
+        <v>0.9</v>
+      </c>
+      <c r="AK12">
+        <v>-0.9</v>
+      </c>
+      <c r="AL12">
+        <v>0.9</v>
       </c>
       <c r="AM12">
         <v>5.9</v>
@@ -1899,7 +2091,7 @@
         <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C13">
         <v>4.5</v>
@@ -1911,7 +2103,7 @@
         <v>-107</v>
       </c>
       <c r="F13" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G13">
         <v>824801</v>
@@ -1970,17 +2162,23 @@
       <c r="Y13">
         <v>1.0657</v>
       </c>
+      <c r="Z13">
+        <v>6</v>
+      </c>
       <c r="AA13" t="s">
-        <v>44</v>
+        <v>52</v>
+      </c>
+      <c r="AB13">
+        <v>-1.12</v>
       </c>
       <c r="AC13" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="AD13">
         <v>3.38</v>
       </c>
       <c r="AE13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF13">
         <v>0.1274</v>
@@ -1990,6 +2188,18 @@
       </c>
       <c r="AH13">
         <v>0</v>
+      </c>
+      <c r="AI13">
+        <v>2.62</v>
+      </c>
+      <c r="AJ13">
+        <v>2.62</v>
+      </c>
+      <c r="AK13">
+        <v>2.62</v>
+      </c>
+      <c r="AL13">
+        <v>2.62</v>
       </c>
       <c r="AM13">
         <v>3.38</v>
@@ -2000,7 +2210,7 @@
         <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C14">
         <v>6.5</v>
@@ -2012,7 +2222,7 @@
         <v>-124</v>
       </c>
       <c r="F14" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="G14">
         <v>824394</v>
@@ -2071,17 +2281,23 @@
       <c r="Y14">
         <v>1.0313</v>
       </c>
+      <c r="Z14">
+        <v>10</v>
+      </c>
       <c r="AA14" t="s">
-        <v>44</v>
+        <v>52</v>
+      </c>
+      <c r="AB14">
+        <v>0.09</v>
       </c>
       <c r="AC14" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="AD14">
         <v>6.59</v>
       </c>
       <c r="AE14" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="AF14">
         <v>0.2599</v>
@@ -2091,6 +2307,18 @@
       </c>
       <c r="AH14">
         <v>0</v>
+      </c>
+      <c r="AI14">
+        <v>3.41</v>
+      </c>
+      <c r="AJ14">
+        <v>3.41</v>
+      </c>
+      <c r="AK14">
+        <v>3.41</v>
+      </c>
+      <c r="AL14">
+        <v>3.41</v>
       </c>
       <c r="AM14">
         <v>6.59</v>
@@ -2101,7 +2329,7 @@
         <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C15">
         <v>5.5</v>
@@ -2113,7 +2341,7 @@
         <v>-104</v>
       </c>
       <c r="F15" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="G15">
         <v>824476</v>
@@ -2172,17 +2400,23 @@
       <c r="Y15">
         <v>1.0673</v>
       </c>
+      <c r="Z15">
+        <v>9</v>
+      </c>
       <c r="AA15" t="s">
-        <v>44</v>
+        <v>52</v>
+      </c>
+      <c r="AB15">
+        <v>1.62</v>
       </c>
       <c r="AC15" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD15">
         <v>7.12</v>
       </c>
       <c r="AE15" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="AF15">
         <v>0.2363</v>
@@ -2192,6 +2426,18 @@
       </c>
       <c r="AH15">
         <v>0</v>
+      </c>
+      <c r="AI15">
+        <v>1.88</v>
+      </c>
+      <c r="AJ15">
+        <v>1.88</v>
+      </c>
+      <c r="AK15">
+        <v>1.88</v>
+      </c>
+      <c r="AL15">
+        <v>1.88</v>
       </c>
       <c r="AM15">
         <v>7.12</v>
@@ -2202,7 +2448,7 @@
         <v>39</v>
       </c>
       <c r="B16" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C16">
         <v>6.5</v>
@@ -2214,7 +2460,7 @@
         <v>-134</v>
       </c>
       <c r="F16" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="G16">
         <v>824476</v>
@@ -2273,17 +2519,23 @@
       <c r="Y16">
         <v>0.8863</v>
       </c>
+      <c r="Z16">
+        <v>8</v>
+      </c>
       <c r="AA16" t="s">
-        <v>44</v>
+        <v>52</v>
+      </c>
+      <c r="AB16">
+        <v>-0.99</v>
       </c>
       <c r="AC16" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="AD16">
         <v>5.51</v>
       </c>
       <c r="AE16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF16">
         <v>0.2924</v>
@@ -2293,6 +2545,18 @@
       </c>
       <c r="AH16">
         <v>0</v>
+      </c>
+      <c r="AI16">
+        <v>2.49</v>
+      </c>
+      <c r="AJ16">
+        <v>2.49</v>
+      </c>
+      <c r="AK16">
+        <v>2.49</v>
+      </c>
+      <c r="AL16">
+        <v>2.49</v>
       </c>
       <c r="AM16">
         <v>5.51</v>
@@ -2303,7 +2567,7 @@
         <v>39</v>
       </c>
       <c r="B17" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C17">
         <v>3.5</v>
@@ -2315,13 +2579,13 @@
         <v>-109</v>
       </c>
       <c r="F17" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G17">
         <v>822937</v>
       </c>
       <c r="H17" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="I17">
         <v>4</v>
@@ -2374,17 +2638,23 @@
       <c r="Y17">
         <v>0.88</v>
       </c>
+      <c r="Z17">
+        <v>1</v>
+      </c>
       <c r="AA17" t="s">
         <v>44</v>
       </c>
+      <c r="AB17">
+        <v>-1.26</v>
+      </c>
       <c r="AC17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD17">
         <v>2.24</v>
       </c>
       <c r="AE17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF17">
         <v>0.1688</v>
@@ -2394,6 +2664,18 @@
       </c>
       <c r="AH17">
         <v>0</v>
+      </c>
+      <c r="AI17">
+        <v>-1.24</v>
+      </c>
+      <c r="AJ17">
+        <v>1.24</v>
+      </c>
+      <c r="AK17">
+        <v>-1.24</v>
+      </c>
+      <c r="AL17">
+        <v>1.24</v>
       </c>
       <c r="AM17">
         <v>2.24</v>
@@ -2404,7 +2686,7 @@
         <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C18">
         <v>5.5</v>
@@ -2416,7 +2698,7 @@
         <v>-137</v>
       </c>
       <c r="F18" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G18">
         <v>822937</v>
@@ -2475,17 +2757,23 @@
       <c r="Y18">
         <v>1.0855</v>
       </c>
+      <c r="Z18">
+        <v>5</v>
+      </c>
       <c r="AA18" t="s">
         <v>44</v>
       </c>
+      <c r="AB18">
+        <v>1.53</v>
+      </c>
       <c r="AC18" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="AD18">
         <v>7.03</v>
       </c>
       <c r="AE18" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="AF18">
         <v>0.2842</v>
@@ -2495,6 +2783,18 @@
       </c>
       <c r="AH18">
         <v>0</v>
+      </c>
+      <c r="AI18">
+        <v>-2.03</v>
+      </c>
+      <c r="AJ18">
+        <v>2.03</v>
+      </c>
+      <c r="AK18">
+        <v>-2.03</v>
+      </c>
+      <c r="AL18">
+        <v>2.03</v>
       </c>
       <c r="AM18">
         <v>7.03</v>
@@ -2505,7 +2805,7 @@
         <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C19">
         <v>3.5</v>
@@ -2517,7 +2817,7 @@
         <v>-147</v>
       </c>
       <c r="F19" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="G19">
         <v>824076</v>
@@ -2576,17 +2876,23 @@
       <c r="Y19">
         <v>0.9044</v>
       </c>
+      <c r="Z19">
+        <v>1</v>
+      </c>
       <c r="AA19" t="s">
         <v>44</v>
       </c>
+      <c r="AB19">
+        <v>-0.71</v>
+      </c>
       <c r="AC19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD19">
         <v>2.79</v>
       </c>
       <c r="AE19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF19">
         <v>0.1562</v>
@@ -2596,6 +2902,18 @@
       </c>
       <c r="AH19">
         <v>0</v>
+      </c>
+      <c r="AI19">
+        <v>-1.79</v>
+      </c>
+      <c r="AJ19">
+        <v>1.79</v>
+      </c>
+      <c r="AK19">
+        <v>-1.79</v>
+      </c>
+      <c r="AL19">
+        <v>1.79</v>
       </c>
       <c r="AM19">
         <v>2.79</v>
@@ -2606,7 +2924,7 @@
         <v>39</v>
       </c>
       <c r="B20" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C20">
         <v>4.5</v>
@@ -2618,7 +2936,7 @@
         <v>-150</v>
       </c>
       <c r="F20" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="G20">
         <v>824076</v>
@@ -2677,17 +2995,23 @@
       <c r="Y20">
         <v>1.0355</v>
       </c>
+      <c r="Z20">
+        <v>3</v>
+      </c>
       <c r="AA20" t="s">
         <v>44</v>
       </c>
+      <c r="AB20">
+        <v>-0.61</v>
+      </c>
       <c r="AC20" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="AD20">
         <v>3.89</v>
       </c>
       <c r="AE20" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF20">
         <v>0.1732</v>
@@ -2697,6 +3021,18 @@
       </c>
       <c r="AH20">
         <v>0</v>
+      </c>
+      <c r="AI20">
+        <v>-0.89</v>
+      </c>
+      <c r="AJ20">
+        <v>0.89</v>
+      </c>
+      <c r="AK20">
+        <v>-0.89</v>
+      </c>
+      <c r="AL20">
+        <v>0.89</v>
       </c>
       <c r="AM20">
         <v>3.89</v>
@@ -2707,7 +3043,7 @@
         <v>39</v>
       </c>
       <c r="B21" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C21">
         <v>6.5</v>
@@ -2719,7 +3055,7 @@
         <v>-137</v>
       </c>
       <c r="F21" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="G21">
         <v>823748</v>
@@ -2778,17 +3114,23 @@
       <c r="Y21">
         <v>0.975</v>
       </c>
+      <c r="Z21">
+        <v>5</v>
+      </c>
       <c r="AA21" t="s">
         <v>44</v>
       </c>
+      <c r="AB21">
+        <v>-0.27</v>
+      </c>
       <c r="AC21" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="AD21">
         <v>6.23</v>
       </c>
       <c r="AE21" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="AF21">
         <v>0.2678</v>
@@ -2798,6 +3140,18 @@
       </c>
       <c r="AH21">
         <v>0</v>
+      </c>
+      <c r="AI21">
+        <v>-1.23</v>
+      </c>
+      <c r="AJ21">
+        <v>1.23</v>
+      </c>
+      <c r="AK21">
+        <v>-1.23</v>
+      </c>
+      <c r="AL21">
+        <v>1.23</v>
       </c>
       <c r="AM21">
         <v>6.23</v>
@@ -2808,7 +3162,7 @@
         <v>39</v>
       </c>
       <c r="B22" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C22">
         <v>5.5</v>
@@ -2820,7 +3174,7 @@
         <v>-135</v>
       </c>
       <c r="F22" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="G22">
         <v>823748</v>
@@ -2879,17 +3233,23 @@
       <c r="Y22">
         <v>0.9742</v>
       </c>
+      <c r="Z22">
+        <v>1</v>
+      </c>
       <c r="AA22" t="s">
         <v>44</v>
       </c>
+      <c r="AB22">
+        <v>-0.72</v>
+      </c>
       <c r="AC22" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD22">
         <v>4.78</v>
       </c>
       <c r="AE22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF22">
         <v>0.2332</v>
@@ -2899,6 +3259,18 @@
       </c>
       <c r="AH22">
         <v>0</v>
+      </c>
+      <c r="AI22">
+        <v>-3.78</v>
+      </c>
+      <c r="AJ22">
+        <v>3.78</v>
+      </c>
+      <c r="AK22">
+        <v>-3.78</v>
+      </c>
+      <c r="AL22">
+        <v>3.78</v>
       </c>
       <c r="AM22">
         <v>4.78</v>
@@ -2909,7 +3281,7 @@
         <v>39</v>
       </c>
       <c r="B23" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C23">
         <v>5.5</v>
@@ -2921,7 +3293,7 @@
         <v>125</v>
       </c>
       <c r="F23" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="G23">
         <v>822860</v>
@@ -2980,17 +3352,23 @@
       <c r="Y23">
         <v>1.0139</v>
       </c>
+      <c r="Z23">
+        <v>11</v>
+      </c>
       <c r="AA23" t="s">
-        <v>44</v>
+        <v>52</v>
+      </c>
+      <c r="AB23">
+        <v>1.21</v>
       </c>
       <c r="AC23" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD23">
         <v>6.71</v>
       </c>
       <c r="AE23" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="AF23">
         <v>0.26</v>
@@ -3000,6 +3378,18 @@
       </c>
       <c r="AH23">
         <v>0</v>
+      </c>
+      <c r="AI23">
+        <v>4.29</v>
+      </c>
+      <c r="AJ23">
+        <v>4.29</v>
+      </c>
+      <c r="AK23">
+        <v>4.29</v>
+      </c>
+      <c r="AL23">
+        <v>4.29</v>
       </c>
       <c r="AM23">
         <v>6.71</v>
@@ -3010,7 +3400,7 @@
         <v>39</v>
       </c>
       <c r="B24" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C24">
         <v>4.5</v>
@@ -3022,7 +3412,7 @@
         <v>-118</v>
       </c>
       <c r="F24" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="G24">
         <v>822860</v>
@@ -3081,17 +3471,23 @@
       <c r="Y24">
         <v>0.9473</v>
       </c>
+      <c r="Z24">
+        <v>3</v>
+      </c>
       <c r="AA24" t="s">
         <v>44</v>
       </c>
+      <c r="AB24">
+        <v>-0.47</v>
+      </c>
       <c r="AC24" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="AD24">
         <v>4.03</v>
       </c>
       <c r="AE24" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF24">
         <v>0.2149</v>
@@ -3101,6 +3497,18 @@
       </c>
       <c r="AH24">
         <v>0</v>
+      </c>
+      <c r="AI24">
+        <v>-1.03</v>
+      </c>
+      <c r="AJ24">
+        <v>1.03</v>
+      </c>
+      <c r="AK24">
+        <v>-1.03</v>
+      </c>
+      <c r="AL24">
+        <v>1.03</v>
       </c>
       <c r="AM24">
         <v>4.03</v>
@@ -3111,10 +3519,10 @@
         <v>39</v>
       </c>
       <c r="B25" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F25" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G25">
         <v>824155</v>
@@ -3174,16 +3582,16 @@
         <v>0.9671</v>
       </c>
       <c r="AA25" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="AC25" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="AD25">
         <v>4.75</v>
       </c>
       <c r="AE25" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF25">
         <v>0.2244</v>
@@ -3203,7 +3611,7 @@
         <v>39</v>
       </c>
       <c r="B26" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C26">
         <v>4.5</v>
@@ -3215,7 +3623,7 @@
         <v>126</v>
       </c>
       <c r="F26" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="G26">
         <v>824318</v>
@@ -3274,17 +3682,23 @@
       <c r="Y26">
         <v>1.0079</v>
       </c>
+      <c r="Z26">
+        <v>6</v>
+      </c>
       <c r="AA26" t="s">
-        <v>44</v>
+        <v>52</v>
+      </c>
+      <c r="AB26">
+        <v>0.86</v>
       </c>
       <c r="AC26" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD26">
         <v>5.36</v>
       </c>
       <c r="AE26" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF26">
         <v>0.2315</v>
@@ -3294,6 +3708,18 @@
       </c>
       <c r="AH26">
         <v>0</v>
+      </c>
+      <c r="AI26">
+        <v>0.64</v>
+      </c>
+      <c r="AJ26">
+        <v>0.64</v>
+      </c>
+      <c r="AK26">
+        <v>0.64</v>
+      </c>
+      <c r="AL26">
+        <v>0.64</v>
       </c>
       <c r="AM26">
         <v>5.36</v>
@@ -3304,7 +3730,7 @@
         <v>39</v>
       </c>
       <c r="B27" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C27">
         <v>3.5</v>
@@ -3316,7 +3742,7 @@
         <v>122</v>
       </c>
       <c r="F27" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="G27">
         <v>824318</v>
@@ -3375,17 +3801,23 @@
       <c r="Y27">
         <v>0.9455</v>
       </c>
+      <c r="Z27">
+        <v>5</v>
+      </c>
       <c r="AA27" t="s">
-        <v>44</v>
+        <v>52</v>
+      </c>
+      <c r="AB27">
+        <v>0.11</v>
       </c>
       <c r="AC27" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="AD27">
         <v>3.61</v>
       </c>
       <c r="AE27" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF27">
         <v>0.1664</v>
@@ -3395,6 +3827,18 @@
       </c>
       <c r="AH27">
         <v>0</v>
+      </c>
+      <c r="AI27">
+        <v>1.39</v>
+      </c>
+      <c r="AJ27">
+        <v>1.39</v>
+      </c>
+      <c r="AK27">
+        <v>1.39</v>
+      </c>
+      <c r="AL27">
+        <v>1.39</v>
       </c>
       <c r="AM27">
         <v>3.61</v>
@@ -3405,7 +3849,7 @@
         <v>39</v>
       </c>
       <c r="B28" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C28">
         <v>4.5</v>
@@ -3417,31 +3861,31 @@
         <v>105</v>
       </c>
       <c r="F28" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G28" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="H28" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="L28">
         <v>6</v>
       </c>
       <c r="S28" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="V28" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="AA28" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="AC28" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="AE28" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
     </row>
     <row r="29" spans="1:39" x14ac:dyDescent="0.25">
@@ -3449,7 +3893,7 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C29">
         <v>3.5</v>
@@ -3461,31 +3905,31 @@
         <v>180</v>
       </c>
       <c r="F29" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G29" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="H29" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="L29">
         <v>1</v>
       </c>
       <c r="S29" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="V29" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="AA29" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="AC29" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="AE29" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
     </row>
     <row r="30" spans="1:39" x14ac:dyDescent="0.25">
@@ -3493,7 +3937,7 @@
         <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C30">
         <v>4.5</v>
@@ -3508,28 +3952,28 @@
         <v>41</v>
       </c>
       <c r="G30" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="H30" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="L30">
         <v>6</v>
       </c>
       <c r="S30" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="V30" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="AA30" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="AC30" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="AE30" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>